<commit_message>
End of week saves
end of week filesaves
</commit_message>
<xml_diff>
--- a/Design_Docs/Instruction_Word_Table.xlsx
+++ b/Design_Docs/Instruction_Word_Table.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Apex\Projects\RISC-V_Project\sfm_RISC-V\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Apex\Projects\RISC-V_Project\sfm_RISC-V\Design_Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6BC5CEA-46F7-4869-B925-952022FB4104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{DAA87B19-7E53-4FE8-8CCB-2B72675DA490}"/>
+    <workbookView xWindow="45972" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{DAA87B19-7E53-4FE8-8CCB-2B72675DA490}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>

</xml_diff>